<commit_message>
Fix column case sensitivity and add auto-cleanup for pivot table artifacts
</commit_message>
<xml_diff>
--- a/test_data/master_test.xlsx
+++ b/test_data/master_test.xlsx
@@ -428,12 +428,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Short description</t>
+          <t>Short Description</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Primary CI/Application</t>
+          <t>Configuration Item</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>

<commit_message>
Fix mapping for Created column and populate Duration
</commit_message>
<xml_diff>
--- a/test_data/master_test.xlsx
+++ b/test_data/master_test.xlsx
@@ -428,12 +428,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Short Description</t>
+          <t>Short description</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Configuration Item</t>
+          <t>Primary CI/Application</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>